<commit_message>
test(module025): remove source workbook metadata and guard export privacy
</commit_message>
<xml_diff>
--- a/src/backend/ProjectTime.Api/Assets/Templates/Module025StandardGsd.xlsx
+++ b/src/backend/ProjectTime.Api/Assets/Templates/Module025StandardGsd.xlsx
@@ -3,12 +3,6 @@
 <x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <x:workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ussignal.sharepoint.com/sites/AS/Architecture/Client Files/P/Pourdre Valley REA/SYS/Dashboard Migration/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{FDF8A73A-2AC1-1949-8848-7D91E5EEDA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C99FB7E-3AC3-CE46-9407-708213E3E468}"/>
   <x:bookViews>
     <x:workbookView xWindow="0" yWindow="620" windowWidth="29040" windowHeight="17520" tabRatio="823" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>

</xml_diff>